<commit_message>
Add Exercise 4A insert records and updated Excel tables
</commit_message>
<xml_diff>
--- a/Xharra_Ex3A_tables.xlsx
+++ b/Xharra_Ex3A_tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arber\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41D89454-0D54-453C-B60B-63C0C3618645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{724DD48C-3D2C-4317-A3F7-2A94C93E46A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" activeTab="3" xr2:uid="{A7CDD78F-32F9-4051-925E-79C7A818BBF1}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>Customer_ID</t>
   </si>
@@ -81,16 +81,45 @@
   </si>
   <si>
     <t>Duration_Minutes</t>
+  </si>
+  <si>
+    <t>John Smith</t>
+  </si>
+  <si>
+    <t>555-123-4567</t>
+  </si>
+  <si>
+    <t>john.smith@example.com</t>
+  </si>
+  <si>
+    <t>123 Main Street, New York, NY</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>Labrador</t>
+  </si>
+  <si>
+    <t>10:AM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -125,8 +154,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -136,13 +166,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -475,10 +510,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E172F3B-92BF-40BD-A3CC-FB582013E1A7}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="9" width="15.6328125" customWidth="1"/>
+    <col min="1" max="5" width="25.6328125" customWidth="1"/>
+    <col min="6" max="9" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -498,35 +534,79 @@
         <v>4</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{1746771B-B30C-4240-B2D7-8FC15BF32ACD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAFA6ABE-BFE8-46B7-892D-CC45EADFC4DE}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="7" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -535,7 +615,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFC5D63A-BC65-441B-BF5F-1B52C3976EF6}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="8" width="15.6328125" customWidth="1"/>
@@ -555,6 +635,24 @@
         <v>12</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1"/>
+      <c r="B2" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -562,17 +660,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDC95BC1-7192-4D98-8DD6-563E40336AFE}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="8" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="1"/>
@@ -580,6 +678,18 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>